<commit_message>
fix(demo): date order checked by code, reference numbers never read as figures
On the VAJRA case the model wrote 'paid on 25 March 2026, which is after the inspection of 2 April
2026' and the verifier passed it - both dates were on the cited lines. The order of two dates is now
checked by code after every verifier (intelligence/chronology.py): a false order is CONTRADICTED,
with the computed order as the reason. The figure reader no longer takes the digits of a reference
number (VJR/SO/2026/014, PV-2026-0356) for amounts: a correct overpayment finding was discarded
because '014' was demanded of the ledger line. The VAJRA ledger now states INR 4,20,00,000 (it held
ten times that), and scripts/demo/run_demo_case.py drives a demonstration case through the API.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/.agent/fixtures/documents/vajra_payment_ledger.xlsx
+++ b/.agent/fixtures/documents/vajra_payment_ledger.xlsx
@@ -469,8 +469,10 @@
           <t>SO/2026/009</t>
         </is>
       </c>
-      <c r="E2" t="n">
-        <v>240000</v>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2,40,000</t>
+        </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -499,8 +501,10 @@
           <t>Invoice TOI/2026/088</t>
         </is>
       </c>
-      <c r="E3" t="n">
-        <v>420000000</v>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>4,20,00,000</t>
+        </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>

</xml_diff>